<commit_message>
fix: 컬러그램 IMD 26.09.07 반영 (v8 77건 → 103건)
v8의 컬러그램 77건이 최신 103건의 부분집합이었음(URL 대조, v8 단독 건 0)
- 컬러그램: 조회수 +68% / 광고비 3.1배 / 매출 2.2배 / 원고료 +6,250,000
- 컬러그램 CPV 36.22 → 25.46원, CPE 5,320 → 4,650원, ER 0.68% → 0.55%
  (필리밀리 4,564원과 사실상 동일 → "국내 CPE 최악" 표현 철회)

전체 총계
- 수량 2,139 → 2,165 (KR 1,998 + 글로벌 167) / 성과 집계 2,086 → 2,112
- 조회수 56,612,765 → 57,682,849 / 참여 468,498 → 472,252
- CPV 15.90 → 15.61원 / CPE 1,922 → 1,907원 / 건당 청구액 420,918 → 415,863원
- 광고 소재 582 → 647 / 광고비 267,691,682 → 283,535,305 / 매출 1,420,018,525 → 1,493,045,674
- ROAS 파트너십 544 → 539% / 합산 530 → 527% / CPA 3,409 → 3,269원
- 조회수 분포 모수 2,112 재계산 (5만↑ 271건 12.83%, 1만↑ 766건 36.27%)
- 원고료 492,408,205 → 498,658,205 (비중 55.4%)
- A4-4 신규: 타 브랜드 IMD 최신화 확인 필요

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Po6GEYZVM1ncJCBSngkbPu
</commit_message>
<xml_diff>
--- a/reports/OYPB_브랜드별_시딩_비용_광고성과_260907 HAN.xlsx
+++ b/reports/OYPB_브랜드별_시딩_비용_광고성과_260907 HAN.xlsx
@@ -824,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:O27"/>
+  <dimension ref="B2:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.2"/>
   <cols>
     <col width="8.796875" customWidth="1" style="3" min="1" max="1"/>
@@ -860,7 +860,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>※ 통계 : 25.04 ~ 26.09 · 국내외 전체 2,139건(글로벌 167건 = JP 99 + US 68) · 26.09.07 기준</t>
+          <t>※ 통계 : 25.04 ~ 26.09 · 국내외 전체 2,165건(글로벌 167건 = JP 99 + US 68) · 26.09.07 기준</t>
         </is>
       </c>
       <c r="C3" s="2" t="n"/>
@@ -879,7 +879,7 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>※ RD : 표준 기준 ⑤ — 수량·비용 전체 2,139건 / 조회수·참여 성과 집계분 2,086건 · 모든 단가는 세금계산서 발행 비용 기준</t>
+          <t>※ RD : 표준 기준 ⑤ — 수량·비용 전체 2,165건 / 조회수·참여 성과 집계분 2,112건 · 모든 단가는 세금계산서 발행 비용 기준</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="O8" s="44" t="n">
-        <v>329997090</v>
+        <v>325861024</v>
       </c>
     </row>
     <row r="9" ht="26.4" customHeight="1" s="35">
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="O9" s="44" t="n">
-        <v>117186968</v>
+        <v>115718190</v>
       </c>
     </row>
     <row r="10" ht="26.4" customHeight="1" s="35">
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="O10" s="44" t="n">
-        <v>108791220</v>
+        <v>107427671</v>
       </c>
     </row>
     <row r="11" ht="39.6" customHeight="1" s="35">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="O11" s="44" t="n">
-        <v>66989232</v>
+        <v>66149614</v>
       </c>
     </row>
     <row r="12" ht="39.6" customHeight="1" s="35">
@@ -1252,7 +1252,7 @@
         <v/>
       </c>
       <c r="H12" s="42" t="n">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="I12" s="43">
         <f>O12/F12</f>
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="O12" s="44" t="n">
-        <v>2944636</v>
+        <v>2907729</v>
       </c>
     </row>
     <row r="13" ht="39.6" customHeight="1" s="35">
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="O14" s="44" t="n">
-        <v>57426917</v>
+        <v>56707149</v>
       </c>
     </row>
     <row r="15" ht="39.6" customHeight="1" s="35">
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="O15" s="44" t="n">
-        <v>68676009</v>
+        <v>67815249</v>
       </c>
     </row>
     <row r="16" ht="39.6" customHeight="1" s="35">
@@ -1498,7 +1498,7 @@
         </is>
       </c>
       <c r="O16" s="44" t="n">
-        <v>39769333</v>
+        <v>39270879</v>
       </c>
     </row>
     <row r="17" ht="39.6" customHeight="1" s="35">
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="C17" s="42" t="n">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="D17" s="42" t="n">
         <v>32</v>
@@ -1518,14 +1518,14 @@
         <v/>
       </c>
       <c r="F17" s="42" t="n">
-        <v>1583237</v>
+        <v>2653321</v>
       </c>
       <c r="G17" s="42">
         <f>F17/E17</f>
         <v/>
       </c>
       <c r="H17" s="42" t="n">
-        <v>10780</v>
+        <v>14526</v>
       </c>
       <c r="I17" s="43">
         <f>O17/F17</f>
@@ -1536,10 +1536,10 @@
         <v/>
       </c>
       <c r="K17" s="42" t="n">
-        <v>7670607</v>
+        <v>23514230</v>
       </c>
       <c r="L17" s="42" t="n">
-        <v>61405809</v>
+        <v>134432958</v>
       </c>
       <c r="M17" s="15">
         <f>L17/K17</f>
@@ -1547,12 +1547,12 @@
       </c>
       <c r="N17" s="16" t="inlineStr">
         <is>
-          <t>전체 브랜드 중 ROAS 2위(800% 이상)
-→ 협업 수량 증가 필요</t>
+          <t>IMD 26.09.07로 103건 확정(v8 77건 → +26)
+조회수 +68% · 광고비 3.1배 · 매출 2.2배</t>
         </is>
       </c>
       <c r="O17" s="44" t="n">
-        <v>57352548</v>
+        <v>67542290</v>
       </c>
     </row>
     <row r="18" ht="39.6" customHeight="1" s="35">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="O18" s="44" t="n">
-        <v>6539846</v>
+        <v>6457878</v>
       </c>
     </row>
     <row r="19" ht="39.6" customHeight="1" s="35">
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="O19" s="44" t="n">
-        <v>11135413</v>
+        <v>10995846</v>
       </c>
     </row>
     <row r="20" ht="26.4" customHeight="1" s="35">
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="O20" s="44" t="n">
-        <v>3535052</v>
+        <v>3490745</v>
       </c>
     </row>
     <row r="21" ht="26.4" customHeight="1" s="35">
@@ -1795,14 +1795,14 @@
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>※ 평균 CPV = 세금계산서 ÷ 조회수 / 평균 CPE = 세금계산서 ÷ 참여수 / 참여수 = 좋아요 + 댓글 → 소계 CPV 15.90원 · CPE 1,922원 · 건당 청구액 420,918원</t>
+          <t>※ 평균 CPV = 세금계산서 ÷ 조회수 / 평균 CPE = 세금계산서 ÷ 참여수 / 참여수 = 좋아요 + 댓글 → 소계 CPV 15.61원 · CPE 1,907원 · 건당 청구액 415,863원</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>※ 참여수는 좋아요 데이터 공란 505건(IMD 2,050건의 24.6%)을 브랜드·국가별 좋아요율과 좋아요/댓글비의 중앙값으로 추정해 반영한 값이다 — 좋아요 실측 358,615 + 추정 78,128 = 436,743, 댓글 31,755(전량 실측)</t>
+          <t>※ 참여수는 좋아요 데이터 공란 519건(IMD 2,076건의 25.0%)을 브랜드·국가별 좋아요율과 좋아요/댓글비의 중앙값으로 추정해 반영한 값이다 — 좋아요 실측 359,877 + 추정 80,292 = 440,169, 댓글 32,083(전량 실측)</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,14 @@
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>※ (참고) 크리에이터 원고료 492,408,205원 = 청구액의 54.7%. 마크업·VAT·솔루션·지급대행 제외 금액으로 위 단가 산정에는 사용하지 않았다.</t>
+          <t>※ (참고) 크리에이터 원고료 498,658,205원 = 청구액의 55.4%. 마크업·VAT·솔루션·지급대행 제외 금액으로 위 단가 산정에는 사용하지 않았다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>※ 컬러그램은 IMD 26.09.07 최신본으로 103건 확정(v8 77건은 부분집합, URL 대조 확인). 다른 브랜드도 동일 누락 가능성이 있어 최신 IMD 확인이 필요하다.</t>
         </is>
       </c>
     </row>

</xml_diff>